<commit_message>
feat: add one example to the codelist template
</commit_message>
<xml_diff>
--- a/codelijst-template.xlsx
+++ b/codelijst-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vandenbrouckekristof/Documents/uncapped/digitaal_vlaanderen/OSLO-codelijsten-generator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39CAE19E-89FC-4D4B-B22A-E323FBEFF0E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99BC3933-C9AD-F745-B078-DBD5B1B8A410}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="16680" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="16680" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="codelijst" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="13">
   <si>
     <t>@id</t>
   </si>
@@ -47,6 +47,24 @@
   </si>
   <si>
     <t>notation</t>
+  </si>
+  <si>
+    <t>https://example.org/id/concept/SchemeA/Concept1</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/2004/02/skos/core#Concept</t>
+  </si>
+  <si>
+    <t>Concept 1</t>
+  </si>
+  <si>
+    <t>First concept in Scheme A</t>
+  </si>
+  <si>
+    <t>https://example.org/id/conceptscheme/SchemeA</t>
+  </si>
+  <si>
+    <t>C1</t>
   </si>
 </sst>
 </file>
@@ -209,7 +227,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="42.6640625" customWidth="1"/>
@@ -243,6 +261,29 @@
         <v>6</v>
       </c>
     </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
@@ -255,7 +296,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77BC371A-FD4C-EB44-8C96-587FE309B299}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.15">
@@ -281,6 +322,29 @@
         <v>6</v>
       </c>
     </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>